<commit_message>
DG Speed Tuning analysis
New analysis files, table template, dataset, and runner.
</commit_message>
<xml_diff>
--- a/result_table_templates/DG_speed_tuning_by_cell.xlsx
+++ b/result_table_templates/DG_speed_tuning_by_cell.xlsx
@@ -1,115 +1,165 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gregschwartz/matlab/DJ_schwartzlab/result_table_templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/augustshin/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3004C9DC-CEAD-5E4E-874D-B7E1ABEF0CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{96110ABB-41CB-1647-9576-0C4DC39CE952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12120" yWindow="500" windowWidth="38060" windowHeight="29520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14980" yWindow="660" windowWidth="14420" windowHeight="18460" xr2:uid="{D12FAE32-61B3-1844-AA2C-FDDC19AADC3F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="181029"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
   <si>
     <t>Field</t>
   </si>
   <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
     <t>file_name</t>
   </si>
   <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>file name from symphony</t>
+  </si>
+  <si>
+    <t>dataset_name</t>
+  </si>
+  <si>
+    <t>dataset name</t>
+  </si>
+  <si>
     <t>source_id</t>
   </si>
   <si>
+    <t>uint16</t>
+  </si>
+  <si>
+    <t>source id used to identify the cell to which the dataset belongs</t>
+  </si>
+  <si>
     <t>speeds</t>
   </si>
   <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>cell</t>
   </si>
   <si>
-    <t>cell</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>set of speeds (microns / sec)</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>max_cycle_avg_amplitude</t>
-  </si>
-  <si>
-    <t>maximum peak to peak amplitude of cycle average trace (mV)</t>
-  </si>
-  <si>
-    <t>mean_cycle_avg_amplitude</t>
-  </si>
-  <si>
-    <t>mean peak to peak amplitude of cycle average trace across directions (mV)</t>
-  </si>
-  <si>
-    <t>min_cycle_avg_peak_neg</t>
-  </si>
-  <si>
-    <t>minimum negative peak of cycle average trace (mV)</t>
-  </si>
-  <si>
-    <t>mean_cycle_avg_peak_neg</t>
-  </si>
-  <si>
-    <t>mean negative peak of cycle average trace (mV)</t>
-  </si>
-  <si>
-    <t>max_cycle_avg_peak_pos</t>
-  </si>
-  <si>
-    <t>maximum positive peak of cycle average trace (mV)</t>
-  </si>
-  <si>
-    <t>mean positive peak of cycle average trace (mV)</t>
-  </si>
-  <si>
-    <t>mean_cycle_avg_peak_pos</t>
-  </si>
-  <si>
-    <t>uint16</t>
-  </si>
-  <si>
-    <t>source id of cell</t>
-  </si>
-  <si>
-    <t>file name of symphony file</t>
+    <t>set of speeds</t>
+  </si>
+  <si>
+    <t>halfwidths</t>
+  </si>
+  <si>
+    <t>set of cycle (bar) halfwidths (microns)</t>
+  </si>
+  <si>
+    <t>contrasts</t>
+  </si>
+  <si>
+    <t>set of contrasts</t>
+  </si>
+  <si>
+    <t>speed_by_condition</t>
+  </si>
+  <si>
+    <t>speed for each condition</t>
+  </si>
+  <si>
+    <t>halfwidth_by_condition</t>
+  </si>
+  <si>
+    <t>halfwidth for each condition</t>
+  </si>
+  <si>
+    <t>contrast_by_condition</t>
+  </si>
+  <si>
+    <t>contrast for each condition</t>
+  </si>
+  <si>
+    <t>preferred_angle_by_condition</t>
+  </si>
+  <si>
+    <t>preferred angle for each condition</t>
+  </si>
+  <si>
+    <t>preferred_orientation_by_condition</t>
+  </si>
+  <si>
+    <t>preferred orientation for each condition</t>
+  </si>
+  <si>
+    <t>dsi_by_condition</t>
+  </si>
+  <si>
+    <t>direction selectivity index for each condition</t>
+  </si>
+  <si>
+    <t>osi_by_condition</t>
+  </si>
+  <si>
+    <t>orientation selectivity index for each condition</t>
+  </si>
+  <si>
+    <t>peak_pref_angle_magnitude_by_condition</t>
+  </si>
+  <si>
+    <t>magnitude at most responsive angle for each condition</t>
+  </si>
+  <si>
+    <t>peak_avg_magnitude_by_condition</t>
+  </si>
+  <si>
+    <t>magnitude averaged across all directions</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -132,9 +182,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -163,39 +212,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -247,7 +296,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -358,13 +407,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -373,6 +415,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -437,24 +486,62 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{6649D996-6833-C548-BBDE-C83189B87AE7}">
+  <we:reference id="93533c7f-4dc5-468f-aba4-1c008e1a7ac8" version="1.0.0.8" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200003101" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9575A2DA-6427-4442-B0AB-B1949B4572BE}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.5" customWidth="1"/>
-    <col min="2" max="2" width="7.5" customWidth="1"/>
-    <col min="3" max="3" width="56.5" customWidth="1"/>
+    <col min="1" max="1" width="35.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -462,113 +549,178 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>